<commit_message>
Add 0930 records and split 核心備份模塊 into its own block
- Add 2026-09-30 records from Sheet_ori.xlsx; every item now carries
  historyDates so the page nav lists both 0926 and 0930 filters
- Apply revised 0926 data: 一般彈匣選擇箱 renamed to 彈匣選擇箱 and the
  2205000000 record moved there from 超彈匣魔方
- Pull all 核心備份模塊 items out of the tiers into a new block shown
  above 層級一, merging entries of the same quantity regardless of the
  [阿利爾] prefix (1/3/5/7/10/15/20個)
- Stats "層級" count excludes the new block
- Sync Sheet.xlsx (歷史成交總集, 0926紀錄, new 0930紀錄 sheet)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -10,6 +10,7 @@
     <sheet name="List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="歷史成交總集" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="0926紀錄" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="0930紀錄" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -451,6 +452,23 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2059,7 +2077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="40.5703125" customWidth="1" style="10" min="1" max="1"/>
@@ -2160,8 +2178,33 @@
       <c r="I4" s="56" t="n">
         <v>1276281562</v>
       </c>
-      <c r="J4" s="56" t="n"/>
-      <c r="K4" s="56" t="n"/>
+      <c r="J4" s="56" t="n">
+        <v>1736437500</v>
+      </c>
+      <c r="K4" s="56" t="n">
+        <v>926100000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>840000000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>525000000</v>
+      </c>
+      <c r="N4" t="n">
+        <v>292526061</v>
+      </c>
+      <c r="O4" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="P4" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>765768937</v>
+      </c>
+      <c r="R4" t="n">
+        <v>347287500</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="10">
       <c r="A5" s="3" t="inlineStr">
@@ -2180,8 +2223,12 @@
       <c r="D5" s="43" t="n">
         <v>1039464085</v>
       </c>
-      <c r="E5" s="56" t="n"/>
-      <c r="F5" s="56" t="n"/>
+      <c r="E5" s="56" t="n">
+        <v>121550625</v>
+      </c>
+      <c r="F5" s="56" t="n">
+        <v>513781804</v>
+      </c>
       <c r="G5" s="56" t="n"/>
       <c r="H5" s="56" t="n"/>
       <c r="I5" s="56" t="n"/>
@@ -2211,11 +2258,21 @@
       <c r="F6" s="56" t="n">
         <v>893397093</v>
       </c>
-      <c r="G6" s="56" t="n"/>
-      <c r="H6" s="56" t="n"/>
-      <c r="I6" s="56" t="n"/>
-      <c r="J6" s="56" t="n"/>
-      <c r="K6" s="56" t="n"/>
+      <c r="G6" s="56" t="n">
+        <v>752456250</v>
+      </c>
+      <c r="H6" s="56" t="n">
+        <v>752456250</v>
+      </c>
+      <c r="I6" s="56" t="n">
+        <v>814447312</v>
+      </c>
+      <c r="J6" s="56" t="n">
+        <v>703550211</v>
+      </c>
+      <c r="K6" s="56" t="n">
+        <v>315000000</v>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="10">
       <c r="A7" s="3" t="inlineStr">
@@ -2234,9 +2291,15 @@
       <c r="D7" s="43" t="n">
         <v>252000000</v>
       </c>
-      <c r="E7" s="56" t="n"/>
-      <c r="F7" s="56" t="n"/>
-      <c r="G7" s="56" t="n"/>
+      <c r="E7" s="56" t="n">
+        <v>52500000</v>
+      </c>
+      <c r="F7" s="56" t="n">
+        <v>231525000</v>
+      </c>
+      <c r="G7" s="56" t="n">
+        <v>115762500</v>
+      </c>
       <c r="H7" s="56" t="n"/>
       <c r="I7" s="56" t="n"/>
       <c r="J7" s="56" t="n"/>
@@ -2256,14 +2319,51 @@
         <f>MAX(D8:K8)</f>
         <v/>
       </c>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="56" t="n"/>
-      <c r="F8" s="56" t="n"/>
-      <c r="G8" s="56" t="n"/>
-      <c r="H8" s="56" t="n"/>
-      <c r="I8" s="56" t="n"/>
-      <c r="J8" s="56" t="n"/>
-      <c r="K8" s="56" t="n"/>
+      <c r="D8" s="43" t="n">
+        <v>15513279</v>
+      </c>
+      <c r="E8" s="56" t="n">
+        <v>231525000</v>
+      </c>
+      <c r="F8" s="56" t="n">
+        <v>17103389</v>
+      </c>
+      <c r="G8" s="56" t="n">
+        <v>32250982</v>
+      </c>
+      <c r="H8" s="56" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="I8" s="56" t="n">
+        <v>20789274</v>
+      </c>
+      <c r="J8" s="56" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="K8" s="56" t="n">
+        <v>26594196</v>
+      </c>
+      <c r="L8" t="n">
+        <v>26250000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>11025000</v>
+      </c>
+      <c r="O8" t="n">
+        <v>13400955</v>
+      </c>
+      <c r="P8" t="n">
+        <v>11576250</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>12249999</v>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="10">
       <c r="A9" s="3" t="inlineStr">
@@ -2285,8 +2385,12 @@
       <c r="E9" s="56" t="n">
         <v>1100000000</v>
       </c>
-      <c r="F9" s="56" t="n"/>
-      <c r="G9" s="56" t="n"/>
+      <c r="F9" s="56" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="G9" s="56" t="n">
+        <v>630000000</v>
+      </c>
       <c r="H9" s="56" t="n"/>
       <c r="I9" s="56" t="n"/>
       <c r="J9" s="56" t="n"/>
@@ -2312,7 +2416,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>一般彈匣選擇箱</t>
+          <t>彈匣選擇箱</t>
         </is>
       </c>
       <c r="B11" s="43">
@@ -2323,10 +2427,18 @@
         <f>MAX(D11:K11)</f>
         <v/>
       </c>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="56" t="n"/>
-      <c r="F11" s="56" t="n"/>
-      <c r="G11" s="56" t="n"/>
+      <c r="D11" s="43" t="n">
+        <v>2205000000</v>
+      </c>
+      <c r="E11" s="56" t="n">
+        <v>2756250000</v>
+      </c>
+      <c r="F11" s="56" t="n">
+        <v>711134520</v>
+      </c>
+      <c r="G11" s="56" t="n">
+        <v>551250000</v>
+      </c>
       <c r="H11" s="56" t="n"/>
       <c r="I11" s="56" t="n"/>
       <c r="J11" s="56" t="n"/>
@@ -2352,11 +2464,21 @@
       <c r="E12" s="56" t="n">
         <v>670000000</v>
       </c>
-      <c r="F12" s="56" t="n"/>
-      <c r="G12" s="56" t="n"/>
-      <c r="H12" s="56" t="n"/>
-      <c r="I12" s="56" t="n"/>
-      <c r="J12" s="56" t="n"/>
+      <c r="F12" s="56" t="n">
+        <v>2625000000</v>
+      </c>
+      <c r="G12" s="56" t="n">
+        <v>1914422343</v>
+      </c>
+      <c r="H12" s="56" t="n">
+        <v>718342527</v>
+      </c>
+      <c r="I12" s="56" t="n">
+        <v>620531284</v>
+      </c>
+      <c r="J12" s="56" t="n">
+        <v>1000000000</v>
+      </c>
       <c r="K12" s="56" t="n"/>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="10">
@@ -2388,9 +2510,30 @@
       <c r="H13" s="56" t="n">
         <v>1215506250</v>
       </c>
-      <c r="I13" s="56" t="n"/>
-      <c r="J13" s="56" t="n"/>
-      <c r="K13" s="56" t="n"/>
+      <c r="I13" s="56" t="n">
+        <v>1181964353</v>
+      </c>
+      <c r="J13" s="56" t="n">
+        <v>1340095640</v>
+      </c>
+      <c r="K13" s="56" t="n">
+        <v>1276281562</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1200000000</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1466005160</v>
+      </c>
+      <c r="N13" t="n">
+        <v>2205000000</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1000637680</v>
+      </c>
+      <c r="P13" t="n">
+        <v>630000000</v>
+      </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="10">
       <c r="A14" s="3" t="inlineStr">
@@ -2415,11 +2558,27 @@
       <c r="F14" s="56" t="n">
         <v>1215506250</v>
       </c>
-      <c r="G14" s="56" t="n"/>
-      <c r="H14" s="56" t="n"/>
-      <c r="I14" s="56" t="n"/>
-      <c r="J14" s="56" t="n"/>
-      <c r="K14" s="56" t="n"/>
+      <c r="G14" s="56" t="n">
+        <v>240661916</v>
+      </c>
+      <c r="H14" s="56" t="n">
+        <v>700000000</v>
+      </c>
+      <c r="I14" s="56" t="n">
+        <v>565694738</v>
+      </c>
+      <c r="J14" s="56" t="n">
+        <v>525000000</v>
+      </c>
+      <c r="K14" s="56" t="n">
+        <v>989965796</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1155000000</v>
+      </c>
+      <c r="M14" t="n">
+        <v>140710041</v>
+      </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="10">
       <c r="A15" s="3" t="inlineStr">
@@ -2435,8 +2594,12 @@
         <f>MAX(D15:K15)</f>
         <v/>
       </c>
-      <c r="D15" s="43" t="n"/>
-      <c r="E15" s="56" t="n"/>
+      <c r="D15" s="43" t="n">
+        <v>36465187</v>
+      </c>
+      <c r="E15" s="56" t="n">
+        <v>136500000</v>
+      </c>
       <c r="F15" s="56" t="n"/>
       <c r="G15" s="56" t="n"/>
       <c r="H15" s="56" t="n"/>
@@ -2496,13 +2659,27 @@
       <c r="D17" s="43" t="n">
         <v>864388452</v>
       </c>
-      <c r="E17" s="56" t="n"/>
-      <c r="F17" s="56" t="n"/>
-      <c r="G17" s="56" t="n"/>
-      <c r="H17" s="56" t="n"/>
-      <c r="I17" s="56" t="n"/>
-      <c r="J17" s="56" t="n"/>
-      <c r="K17" s="56" t="n"/>
+      <c r="E17" s="56" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="F17" s="56" t="n">
+        <v>638140781</v>
+      </c>
+      <c r="G17" s="56" t="n">
+        <v>945000000</v>
+      </c>
+      <c r="H17" s="56" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="I17" s="56" t="n">
+        <v>3257789252</v>
+      </c>
+      <c r="J17" s="56" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="K17" s="56" t="n">
+        <v>926100000</v>
+      </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="10">
       <c r="A18" s="2" t="inlineStr">
@@ -2586,7 +2763,7 @@
         <v/>
       </c>
       <c r="D21" s="43" t="n">
-        <v>2205000000</v>
+        <v>4190331415</v>
       </c>
       <c r="E21" s="56" t="n"/>
       <c r="F21" s="56" t="n"/>
@@ -2613,7 +2790,9 @@
       <c r="D22" s="43" t="n">
         <v>3000000000</v>
       </c>
-      <c r="E22" s="56" t="n"/>
+      <c r="E22" s="56" t="n">
+        <v>2814200845</v>
+      </c>
       <c r="F22" s="56" t="n"/>
       <c r="G22" s="56" t="n"/>
       <c r="H22" s="56" t="n"/>
@@ -3039,19 +3218,16 @@
         <f>MAX(D41:K41)</f>
         <v/>
       </c>
-      <c r="D41" s="43">
-        <f>G41</f>
-        <v/>
-      </c>
-      <c r="E41" s="56">
-        <f>E16*10</f>
-        <v/>
-      </c>
-      <c r="F41" s="56" t="n"/>
-      <c r="G41" s="56">
-        <f>G16*10</f>
-        <v/>
-      </c>
+      <c r="D41" s="43" t="n">
+        <v>3307500000</v>
+      </c>
+      <c r="E41" s="56" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="F41" s="56" t="n">
+        <v>3307500000</v>
+      </c>
+      <c r="G41" s="56" t="n"/>
       <c r="H41" s="56" t="n"/>
       <c r="I41" s="56" t="n"/>
       <c r="J41" s="56" t="n"/>
@@ -3528,7 +3704,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>一般彈匣選擇箱</t>
+          <t>彈匣選擇箱</t>
         </is>
       </c>
       <c r="B11" s="43">
@@ -3539,7 +3715,9 @@
         <f>MAX(D11:K11)</f>
         <v/>
       </c>
-      <c r="D11" s="43" t="n"/>
+      <c r="D11" s="43" t="n">
+        <v>2205000000</v>
+      </c>
       <c r="E11" s="56" t="n"/>
       <c r="F11" s="56" t="n"/>
       <c r="G11" s="56" t="n"/>
@@ -3801,9 +3979,7 @@
         <f>MAX(D21:K21)</f>
         <v/>
       </c>
-      <c r="D21" s="43" t="n">
-        <v>2205000000</v>
-      </c>
+      <c r="D21" s="43" t="n"/>
       <c r="E21" s="56" t="n"/>
       <c r="F21" s="56" t="n"/>
       <c r="G21" s="56" t="n"/>
@@ -4255,19 +4431,16 @@
         <f>MAX(D41:K41)</f>
         <v/>
       </c>
-      <c r="D41" s="43">
-        <f>G41</f>
-        <v/>
-      </c>
-      <c r="E41" s="56">
-        <f>E16*10</f>
-        <v/>
-      </c>
-      <c r="F41" s="56" t="n"/>
-      <c r="G41" s="56">
-        <f>G16*10</f>
-        <v/>
-      </c>
+      <c r="D41" s="43" t="n">
+        <v>3307500000</v>
+      </c>
+      <c r="E41" s="56" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="F41" s="56" t="n">
+        <v>3307500000</v>
+      </c>
+      <c r="G41" s="56" t="n"/>
       <c r="H41" s="56" t="n"/>
       <c r="I41" s="56" t="n"/>
       <c r="J41" s="56" t="n"/>
@@ -4471,4 +4644,1289 @@
   <pageSetup orientation="portrait" paperSize="9"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <cols>
+    <col width="40.5703125" customWidth="1" style="10" min="1" max="1"/>
+    <col width="19.85546875" customWidth="1" style="10" min="2" max="2"/>
+    <col width="18.5703125" customWidth="1" style="5" min="3" max="3"/>
+    <col width="18.5703125" customWidth="1" style="10" min="4" max="4"/>
+    <col width="16.7109375" customWidth="1" style="10" min="5" max="5"/>
+    <col width="18.28515625" customWidth="1" style="10" min="6" max="6"/>
+    <col width="18.28515625" customWidth="1" style="40" min="7" max="8"/>
+    <col width="18.28515625" customWidth="1" style="10" min="9" max="10"/>
+    <col width="18.140625" customWidth="1" style="10" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>最低價參考</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>最高價參考</t>
+        </is>
+      </c>
+      <c r="D1" s="36" t="inlineStr">
+        <is>
+          <t>成交ED名目紀錄</t>
+        </is>
+      </c>
+      <c r="E1" s="52" t="inlineStr">
+        <is>
+          <t>ED比值</t>
+        </is>
+      </c>
+      <c r="F1" s="40" t="n"/>
+      <c r="H1" t="n"/>
+      <c r="I1" s="40" t="n"/>
+      <c r="J1" s="41" t="n"/>
+      <c r="K1" s="40" t="n"/>
+    </row>
+    <row r="2" ht="16.5" customHeight="1" s="10">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>【黑暗精靈黑市 - 可能出現的拍賣品】</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="D2" s="53" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E2" s="54" t="n">
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="10">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">層級一 </t>
+        </is>
+      </c>
+      <c r="B3" s="48" t="n"/>
+      <c r="C3" s="49" t="n"/>
+      <c r="D3" s="48" t="n"/>
+      <c r="E3" s="55" t="n"/>
+      <c r="F3" s="55" t="n"/>
+      <c r="G3" s="55" t="n"/>
+      <c r="H3" s="55" t="n"/>
+      <c r="I3" s="55" t="n"/>
+      <c r="J3" s="55" t="n"/>
+      <c r="K3" s="55" t="n"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="10">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>一般彈匣魔方</t>
+        </is>
+      </c>
+      <c r="B4" s="43">
+        <f>MIN(D4:K4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="44">
+        <f>MAX(D4:K4)</f>
+        <v/>
+      </c>
+      <c r="D4" s="45" t="n">
+        <v>1736437500</v>
+      </c>
+      <c r="E4" s="56" t="n">
+        <v>926100000</v>
+      </c>
+      <c r="F4" s="56" t="n">
+        <v>840000000</v>
+      </c>
+      <c r="G4" s="56" t="n">
+        <v>525000000</v>
+      </c>
+      <c r="H4" s="56" t="n">
+        <v>292526061</v>
+      </c>
+      <c r="I4" s="56" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="J4" s="56" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="K4" s="56" t="n">
+        <v>765768937</v>
+      </c>
+      <c r="L4" t="n">
+        <v>347287500</v>
+      </c>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="10">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>黑色碎片2個</t>
+        </is>
+      </c>
+      <c r="B5" s="43">
+        <f>MIN(D5:K5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="44">
+        <f>MAX(D5:K5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="43" t="n">
+        <v>121550625</v>
+      </c>
+      <c r="E5" s="56" t="n">
+        <v>513781804</v>
+      </c>
+      <c r="F5" s="56" t="n"/>
+      <c r="G5" s="56" t="n"/>
+      <c r="H5" s="56" t="n"/>
+      <c r="I5" s="56" t="n"/>
+      <c r="J5" s="56" t="n"/>
+      <c r="K5" s="56" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="10">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項轉換石3個</t>
+        </is>
+      </c>
+      <c r="B6" s="43">
+        <f>MIN(D6:K6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="44">
+        <f>MAX(D6:K6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="43" t="n">
+        <v>752456250</v>
+      </c>
+      <c r="E6" s="56" t="n">
+        <v>752456250</v>
+      </c>
+      <c r="F6" s="56" t="n">
+        <v>814447312</v>
+      </c>
+      <c r="G6" s="56" t="n">
+        <v>703550211</v>
+      </c>
+      <c r="H6" s="56" t="n">
+        <v>315000000</v>
+      </c>
+      <c r="I6" s="56" t="n"/>
+      <c r="J6" s="56" t="n"/>
+      <c r="K6" s="56" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="10">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項備份卷1個</t>
+        </is>
+      </c>
+      <c r="B7" s="43">
+        <f>MIN(D7:K7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="44">
+        <f>MAX(D7:K7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="43" t="n">
+        <v>52500000</v>
+      </c>
+      <c r="E7" s="56" t="n">
+        <v>231525000</v>
+      </c>
+      <c r="F7" s="56" t="n">
+        <v>115762500</v>
+      </c>
+      <c r="G7" s="56" t="n"/>
+      <c r="H7" s="56" t="n"/>
+      <c r="I7" s="56" t="n"/>
+      <c r="J7" s="56" t="n"/>
+      <c r="K7" s="56" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="10">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 核心備份模塊1個</t>
+        </is>
+      </c>
+      <c r="B8" s="43">
+        <f>MIN(D8:K8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="44">
+        <f>MAX(D8:K8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="43" t="n">
+        <v>15513279</v>
+      </c>
+      <c r="E8" s="56" t="n">
+        <v>231525000</v>
+      </c>
+      <c r="F8" s="56" t="n">
+        <v>17103389</v>
+      </c>
+      <c r="G8" s="56" t="n">
+        <v>32250982</v>
+      </c>
+      <c r="H8" s="56" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="I8" s="56" t="n">
+        <v>20789274</v>
+      </c>
+      <c r="J8" s="56" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="K8" s="56" t="n">
+        <v>26594196</v>
+      </c>
+      <c r="L8" t="n">
+        <v>26250000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>11025000</v>
+      </c>
+      <c r="O8" t="n">
+        <v>13400955</v>
+      </c>
+      <c r="P8" t="n">
+        <v>11576250</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>12249999</v>
+      </c>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="10">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>每周鍛造材料1000個</t>
+        </is>
+      </c>
+      <c r="B9" s="43">
+        <f>MIN(D9:K9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="44">
+        <f>MAX(D9:K9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E9" s="56" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="F9" s="56" t="n"/>
+      <c r="G9" s="56" t="n"/>
+      <c r="H9" s="56" t="n"/>
+      <c r="I9" s="56" t="n"/>
+      <c r="J9" s="56" t="n"/>
+      <c r="K9" s="56" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">層級二 </t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="n"/>
+      <c r="C10" s="58" t="n"/>
+      <c r="D10" s="48" t="n"/>
+      <c r="E10" s="55" t="n"/>
+      <c r="F10" s="55" t="n"/>
+      <c r="G10" s="55" t="n"/>
+      <c r="H10" s="55" t="n"/>
+      <c r="I10" s="55" t="n"/>
+      <c r="J10" s="55" t="n"/>
+      <c r="K10" s="55" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="10">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>彈匣選擇箱</t>
+        </is>
+      </c>
+      <c r="B11" s="43">
+        <f>MIN(D11:K11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="44">
+        <f>MAX(D11:K11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>2756250000</v>
+      </c>
+      <c r="E11" s="56" t="n">
+        <v>711134520</v>
+      </c>
+      <c r="F11" s="56" t="n">
+        <v>551250000</v>
+      </c>
+      <c r="G11" s="56" t="n"/>
+      <c r="H11" s="56" t="n"/>
+      <c r="I11" s="56" t="n"/>
+      <c r="J11" s="56" t="n"/>
+      <c r="K11" s="56" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="10">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>黑色碎片4個</t>
+        </is>
+      </c>
+      <c r="B12" s="43">
+        <f>MIN(D12:K12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="44">
+        <f>MAX(D12:K12)</f>
+        <v/>
+      </c>
+      <c r="D12" s="43" t="n">
+        <v>2625000000</v>
+      </c>
+      <c r="E12" s="56" t="n">
+        <v>1914422343</v>
+      </c>
+      <c r="F12" s="56" t="n">
+        <v>718342527</v>
+      </c>
+      <c r="G12" s="56" t="n">
+        <v>620531284</v>
+      </c>
+      <c r="H12" s="56" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I12" s="56" t="n"/>
+      <c r="J12" s="56" t="n"/>
+      <c r="K12" s="56" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="10">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項轉換石5個</t>
+        </is>
+      </c>
+      <c r="B13" s="43">
+        <f>MIN(D13:K13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="44">
+        <f>MAX(D13:K13)</f>
+        <v/>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>1181964353</v>
+      </c>
+      <c r="E13" s="56" t="n">
+        <v>1340095640</v>
+      </c>
+      <c r="F13" s="56" t="n">
+        <v>1276281562</v>
+      </c>
+      <c r="G13" s="56" t="n">
+        <v>1200000000</v>
+      </c>
+      <c r="H13" s="56" t="n">
+        <v>1466005160</v>
+      </c>
+      <c r="I13" s="56" t="n">
+        <v>2205000000</v>
+      </c>
+      <c r="J13" s="56" t="n">
+        <v>1000637680</v>
+      </c>
+      <c r="K13" s="56" t="n">
+        <v>630000000</v>
+      </c>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="10">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項備份卷3個</t>
+        </is>
+      </c>
+      <c r="B14" s="43">
+        <f>MIN(D14:K14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="44">
+        <f>MAX(D14:K14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="43" t="n">
+        <v>240661916</v>
+      </c>
+      <c r="E14" s="56" t="n">
+        <v>700000000</v>
+      </c>
+      <c r="F14" s="56" t="n">
+        <v>565694738</v>
+      </c>
+      <c r="G14" s="56" t="n">
+        <v>525000000</v>
+      </c>
+      <c r="H14" s="56" t="n">
+        <v>989965796</v>
+      </c>
+      <c r="I14" s="56" t="n">
+        <v>1155000000</v>
+      </c>
+      <c r="J14" s="56" t="n">
+        <v>140710041</v>
+      </c>
+      <c r="K14" s="56" t="n"/>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="10">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 核心備份模塊3個</t>
+        </is>
+      </c>
+      <c r="B15" s="43">
+        <f>MIN(D15:K15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="44">
+        <f>MAX(D15:K15)</f>
+        <v/>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>36465187</v>
+      </c>
+      <c r="E15" s="56" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="F15" s="56" t="n"/>
+      <c r="G15" s="56" t="n"/>
+      <c r="H15" s="56" t="n"/>
+      <c r="I15" s="56" t="n"/>
+      <c r="J15" s="56" t="n"/>
+      <c r="K15" s="56" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="10">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>核心備份模塊1個</t>
+        </is>
+      </c>
+      <c r="B16" s="43">
+        <f>MIN(D16:K16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="44">
+        <f>MAX(D16:K16)</f>
+        <v/>
+      </c>
+      <c r="D16" s="43" t="n"/>
+      <c r="E16" s="56" t="n"/>
+      <c r="F16" s="56" t="n"/>
+      <c r="G16" s="56" t="n"/>
+      <c r="H16" s="56" t="n"/>
+      <c r="I16" s="56" t="n"/>
+      <c r="J16" s="56" t="n"/>
+      <c r="K16" s="56" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="10">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>每周鍛造材料2000個</t>
+        </is>
+      </c>
+      <c r="B17" s="43">
+        <f>MIN(D17:K17)</f>
+        <v/>
+      </c>
+      <c r="C17" s="44">
+        <f>MAX(D17:K17)</f>
+        <v/>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="E17" s="56" t="n">
+        <v>638140781</v>
+      </c>
+      <c r="F17" s="56" t="n">
+        <v>945000000</v>
+      </c>
+      <c r="G17" s="56" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="H17" s="56" t="n">
+        <v>3257789252</v>
+      </c>
+      <c r="I17" s="56" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="J17" s="56" t="n">
+        <v>926100000</v>
+      </c>
+      <c r="K17" s="56" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="10">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">層級三 </t>
+        </is>
+      </c>
+      <c r="B18" s="57" t="n"/>
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="48" t="n"/>
+      <c r="E18" s="55" t="n"/>
+      <c r="F18" s="55" t="n"/>
+      <c r="G18" s="55" t="n"/>
+      <c r="H18" s="55" t="n"/>
+      <c r="I18" s="55" t="n"/>
+      <c r="J18" s="55" t="n"/>
+      <c r="K18" s="55" t="n"/>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="10">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>核心1個</t>
+        </is>
+      </c>
+      <c r="B19" s="43">
+        <f>MIN(D19:K19)</f>
+        <v/>
+      </c>
+      <c r="C19" s="44">
+        <f>MAX(D19:K19)</f>
+        <v/>
+      </c>
+      <c r="D19" s="43" t="n"/>
+      <c r="E19" s="56" t="n"/>
+      <c r="F19" s="56" t="n"/>
+      <c r="G19" s="56" t="n"/>
+      <c r="H19" s="56" t="n"/>
+      <c r="I19" s="56" t="n"/>
+      <c r="J19" s="56" t="n"/>
+      <c r="K19" s="56" t="n"/>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="10">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 內布隆原型選擇箱</t>
+        </is>
+      </c>
+      <c r="B20" s="43">
+        <f>MIN(D20:K20)</f>
+        <v/>
+      </c>
+      <c r="C20" s="44">
+        <f>MAX(D20:K20)</f>
+        <v/>
+      </c>
+      <c r="D20" s="43" t="n"/>
+      <c r="E20" s="56" t="n"/>
+      <c r="F20" s="56" t="n"/>
+      <c r="G20" s="56" t="n"/>
+      <c r="H20" s="56" t="n"/>
+      <c r="I20" s="56" t="n"/>
+      <c r="J20" s="56" t="n"/>
+      <c r="K20" s="56" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="10">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>超彈匣魔方</t>
+        </is>
+      </c>
+      <c r="B21" s="43">
+        <f>MIN(D21:K21)</f>
+        <v/>
+      </c>
+      <c r="C21" s="44">
+        <f>MAX(D21:K21)</f>
+        <v/>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>4190331415</v>
+      </c>
+      <c r="E21" s="56" t="n"/>
+      <c r="F21" s="56" t="n"/>
+      <c r="G21" s="56" t="n"/>
+      <c r="H21" s="56" t="n"/>
+      <c r="I21" s="56" t="n"/>
+      <c r="J21" s="56" t="n"/>
+      <c r="K21" s="56" t="n"/>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="10">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項轉換石10個</t>
+        </is>
+      </c>
+      <c r="B22" s="43">
+        <f>MIN(D22:K22)</f>
+        <v/>
+      </c>
+      <c r="C22" s="44">
+        <f>MAX(D22:K22)</f>
+        <v/>
+      </c>
+      <c r="D22" s="43" t="n">
+        <v>2814200845</v>
+      </c>
+      <c r="E22" s="56" t="n"/>
+      <c r="F22" s="56" t="n"/>
+      <c r="G22" s="56" t="n"/>
+      <c r="H22" s="56" t="n"/>
+      <c r="I22" s="56" t="n"/>
+      <c r="J22" s="56" t="n"/>
+      <c r="K22" s="56" t="n"/>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="10">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>支援 &amp; 戰鬥 &amp; 通用彈匣選擇箱</t>
+        </is>
+      </c>
+      <c r="B23" s="43">
+        <f>MIN(D23:K23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="44">
+        <f>MAX(D23:K23)</f>
+        <v/>
+      </c>
+      <c r="D23" s="43" t="n"/>
+      <c r="E23" s="56" t="n"/>
+      <c r="F23" s="56" t="n"/>
+      <c r="G23" s="56" t="n"/>
+      <c r="H23" s="56" t="n"/>
+      <c r="I23" s="56" t="n"/>
+      <c r="J23" s="56" t="n"/>
+      <c r="K23" s="56" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="10">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 核心備份模塊10個</t>
+        </is>
+      </c>
+      <c r="B24" s="43">
+        <f>MIN(D24:K24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="44">
+        <f>MAX(D24:K24)</f>
+        <v/>
+      </c>
+      <c r="D24" s="43" t="n"/>
+      <c r="E24" s="56" t="n"/>
+      <c r="F24" s="56" t="n"/>
+      <c r="G24" s="56" t="n"/>
+      <c r="H24" s="56" t="n"/>
+      <c r="I24" s="56" t="n"/>
+      <c r="J24" s="56" t="n"/>
+      <c r="K24" s="56" t="n"/>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="10">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>核心備份模塊5個</t>
+        </is>
+      </c>
+      <c r="B25" s="43">
+        <f>MIN(D25:K25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="44">
+        <f>MAX(D25:K25)</f>
+        <v/>
+      </c>
+      <c r="D25" s="43" t="n"/>
+      <c r="E25" s="56" t="n"/>
+      <c r="F25" s="56" t="n"/>
+      <c r="G25" s="56" t="n"/>
+      <c r="H25" s="56" t="n"/>
+      <c r="I25" s="56" t="n"/>
+      <c r="J25" s="56" t="n"/>
+      <c r="K25" s="56" t="n"/>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="10">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">層級四 </t>
+        </is>
+      </c>
+      <c r="B26" s="57" t="n"/>
+      <c r="C26" s="58" t="n"/>
+      <c r="D26" s="48" t="n"/>
+      <c r="E26" s="55" t="n"/>
+      <c r="F26" s="55" t="n"/>
+      <c r="G26" s="55" t="n"/>
+      <c r="H26" s="55" t="n"/>
+      <c r="I26" s="55" t="n"/>
+      <c r="J26" s="55" t="n"/>
+      <c r="K26" s="55" t="n"/>
+    </row>
+    <row r="27" ht="16.5" customHeight="1" s="10">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>穩定的核心1個</t>
+        </is>
+      </c>
+      <c r="B27" s="43">
+        <f>MIN(D27:K27)</f>
+        <v/>
+      </c>
+      <c r="C27" s="44">
+        <f>MAX(D27:K27)</f>
+        <v/>
+      </c>
+      <c r="D27" s="43" t="n"/>
+      <c r="E27" s="56" t="n"/>
+      <c r="F27" s="56" t="n"/>
+      <c r="G27" s="56" t="n"/>
+      <c r="H27" s="56" t="n"/>
+      <c r="I27" s="56" t="n"/>
+      <c r="J27" s="56" t="n"/>
+      <c r="K27" s="56" t="n"/>
+    </row>
+    <row r="28" ht="16.5" customHeight="1" s="10">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>內布隆原型選擇箱</t>
+        </is>
+      </c>
+      <c r="B28" s="43">
+        <f>MIN(D28:K28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="44">
+        <f>MAX(D28:K28)</f>
+        <v/>
+      </c>
+      <c r="D28" s="43" t="n"/>
+      <c r="E28" s="56" t="n"/>
+      <c r="F28" s="56" t="n"/>
+      <c r="G28" s="56" t="n"/>
+      <c r="H28" s="56" t="n"/>
+      <c r="I28" s="56" t="n"/>
+      <c r="J28" s="56" t="n"/>
+      <c r="K28" s="56" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="10">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>超彈匣選擇箱</t>
+        </is>
+      </c>
+      <c r="B29" s="43">
+        <f>MIN(D29:K29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="44">
+        <f>MAX(D29:K29)</f>
+        <v/>
+      </c>
+      <c r="D29" s="43" t="n"/>
+      <c r="E29" s="56" t="n"/>
+      <c r="F29" s="56" t="n"/>
+      <c r="G29" s="56" t="n"/>
+      <c r="H29" s="56" t="n"/>
+      <c r="I29" s="56" t="n"/>
+      <c r="J29" s="56" t="n"/>
+      <c r="K29" s="56" t="n"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="10">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 1%電路T板選擇箱</t>
+        </is>
+      </c>
+      <c r="B30" s="43">
+        <f>MIN(D30:K30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="44">
+        <f>MAX(D30:K30)</f>
+        <v/>
+      </c>
+      <c r="D30" s="43" t="n"/>
+      <c r="E30" s="56" t="n"/>
+      <c r="F30" s="56" t="n"/>
+      <c r="G30" s="56" t="n"/>
+      <c r="H30" s="56" t="n"/>
+      <c r="I30" s="56" t="n"/>
+      <c r="J30" s="56" t="n"/>
+      <c r="K30" s="56" t="n"/>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="10">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 1%電路L板選擇箱</t>
+        </is>
+      </c>
+      <c r="B31" s="43">
+        <f>MIN(D31:K31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="44">
+        <f>MAX(D31:K31)</f>
+        <v/>
+      </c>
+      <c r="D31" s="43" t="n"/>
+      <c r="E31" s="56" t="n"/>
+      <c r="F31" s="56" t="n"/>
+      <c r="G31" s="56" t="n"/>
+      <c r="H31" s="56" t="n"/>
+      <c r="I31" s="56" t="n"/>
+      <c r="J31" s="56" t="n"/>
+      <c r="K31" s="56" t="n"/>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="10">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項轉換石15個</t>
+        </is>
+      </c>
+      <c r="B32" s="43">
+        <f>MIN(D32:K32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="44">
+        <f>MAX(D32:K32)</f>
+        <v/>
+      </c>
+      <c r="D32" s="43" t="n"/>
+      <c r="E32" s="56" t="n"/>
+      <c r="F32" s="56" t="n"/>
+      <c r="G32" s="56" t="n"/>
+      <c r="H32" s="56" t="n"/>
+      <c r="I32" s="56" t="n"/>
+      <c r="J32" s="56" t="n"/>
+      <c r="K32" s="56" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="10">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 核心備份模塊15個</t>
+        </is>
+      </c>
+      <c r="B33" s="43">
+        <f>MIN(D33:K33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="44">
+        <f>MAX(D33:K33)</f>
+        <v/>
+      </c>
+      <c r="D33" s="43" t="n"/>
+      <c r="E33" s="56" t="n"/>
+      <c r="F33" s="56" t="n"/>
+      <c r="G33" s="56" t="n"/>
+      <c r="H33" s="56" t="n"/>
+      <c r="I33" s="56" t="n"/>
+      <c r="J33" s="56" t="n"/>
+      <c r="K33" s="56" t="n"/>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="10">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>核心備份模塊7個</t>
+        </is>
+      </c>
+      <c r="B34" s="43">
+        <f>MIN(D34:K34)</f>
+        <v/>
+      </c>
+      <c r="C34" s="44">
+        <f>MAX(D34:K34)</f>
+        <v/>
+      </c>
+      <c r="D34" s="43" t="n"/>
+      <c r="E34" s="56" t="n"/>
+      <c r="F34" s="56" t="n"/>
+      <c r="G34" s="56" t="n"/>
+      <c r="H34" s="56" t="n"/>
+      <c r="I34" s="56" t="n"/>
+      <c r="J34" s="56" t="n"/>
+      <c r="K34" s="56" t="n"/>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="10">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">層級五 </t>
+        </is>
+      </c>
+      <c r="B35" s="57" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="48" t="n"/>
+      <c r="E35" s="55" t="n"/>
+      <c r="F35" s="55" t="n"/>
+      <c r="G35" s="55" t="n"/>
+      <c r="H35" s="55" t="n"/>
+      <c r="I35" s="55" t="n"/>
+      <c r="J35" s="55" t="n"/>
+      <c r="K35" s="55" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="10">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 死級詞條升級券1個</t>
+        </is>
+      </c>
+      <c r="B36" s="43">
+        <f>MIN(D36:K36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="44">
+        <f>MAX(D36:K36)</f>
+        <v/>
+      </c>
+      <c r="D36" s="43" t="n"/>
+      <c r="E36" s="56" t="n"/>
+      <c r="F36" s="56" t="n"/>
+      <c r="G36" s="56" t="n"/>
+      <c r="H36" s="56" t="n"/>
+      <c r="I36" s="56" t="n"/>
+      <c r="J36" s="56" t="n"/>
+      <c r="K36" s="56" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="10">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具詞條升級券1個</t>
+        </is>
+      </c>
+      <c r="B37" s="43">
+        <f>MIN(D37:K37)</f>
+        <v/>
+      </c>
+      <c r="C37" s="44">
+        <f>MAX(D37:K37)</f>
+        <v/>
+      </c>
+      <c r="D37" s="43" t="n"/>
+      <c r="E37" s="56" t="n"/>
+      <c r="F37" s="56" t="n"/>
+      <c r="G37" s="56" t="n"/>
+      <c r="H37" s="56" t="n"/>
+      <c r="I37" s="56" t="n"/>
+      <c r="J37" s="56" t="n"/>
+      <c r="K37" s="56" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="10">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 複製電路選擇箱</t>
+        </is>
+      </c>
+      <c r="B38" s="43">
+        <f>MIN(D38:K38)</f>
+        <v/>
+      </c>
+      <c r="C38" s="44">
+        <f>MAX(D38:K38)</f>
+        <v/>
+      </c>
+      <c r="D38" s="43" t="n"/>
+      <c r="E38" s="56" t="n"/>
+      <c r="F38" s="56" t="n"/>
+      <c r="G38" s="56" t="n"/>
+      <c r="H38" s="56" t="n"/>
+      <c r="I38" s="56" t="n"/>
+      <c r="J38" s="56" t="n"/>
+      <c r="K38" s="56" t="n"/>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="10">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 防具選項轉換石20個</t>
+        </is>
+      </c>
+      <c r="B39" s="43">
+        <f>MIN(D39:K39)</f>
+        <v/>
+      </c>
+      <c r="C39" s="44">
+        <f>MAX(D39:K39)</f>
+        <v/>
+      </c>
+      <c r="D39" s="43" t="n"/>
+      <c r="E39" s="56" t="n"/>
+      <c r="F39" s="56" t="n"/>
+      <c r="G39" s="56" t="n"/>
+      <c r="H39" s="56" t="n"/>
+      <c r="I39" s="56" t="n"/>
+      <c r="J39" s="56" t="n"/>
+      <c r="K39" s="56" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="10">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>[阿利爾] 核心備份模塊20個</t>
+        </is>
+      </c>
+      <c r="B40" s="43">
+        <f>MIN(D40:K40)</f>
+        <v/>
+      </c>
+      <c r="C40" s="44">
+        <f>MAX(D40:K40)</f>
+        <v/>
+      </c>
+      <c r="D40" s="43" t="n"/>
+      <c r="E40" s="56" t="n"/>
+      <c r="F40" s="56" t="n"/>
+      <c r="G40" s="56" t="n"/>
+      <c r="H40" s="56" t="n"/>
+      <c r="I40" s="56" t="n"/>
+      <c r="J40" s="56" t="n"/>
+      <c r="K40" s="56" t="n"/>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="10">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>核心備份模塊10個</t>
+        </is>
+      </c>
+      <c r="B41" s="43">
+        <f>MIN(D41:K41)</f>
+        <v/>
+      </c>
+      <c r="C41" s="44">
+        <f>MAX(D41:K41)</f>
+        <v/>
+      </c>
+      <c r="D41" s="43" t="n"/>
+      <c r="E41" s="56" t="n"/>
+      <c r="F41" s="56" t="n"/>
+      <c r="G41" s="56" t="n"/>
+      <c r="H41" s="56" t="n"/>
+      <c r="I41" s="56" t="n"/>
+      <c r="J41" s="56" t="n"/>
+      <c r="K41" s="56" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="10">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="48" t="n"/>
+      <c r="C42" s="49" t="n"/>
+      <c r="D42" s="48" t="n"/>
+      <c r="E42" s="55" t="n"/>
+      <c r="F42" s="55" t="n"/>
+      <c r="G42" s="55" t="n"/>
+      <c r="H42" s="55" t="n"/>
+      <c r="I42" s="55" t="n"/>
+      <c r="J42" s="55" t="n"/>
+      <c r="K42" s="55" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="16" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="16" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="16" t="n"/>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="16" t="n"/>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="16" t="n"/>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="16" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="16" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="16" t="n"/>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="16" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="16" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="16" t="n"/>
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="16" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="16" t="n"/>
+      <c r="C51" s="15" t="n"/>
+      <c r="D51" s="16" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="16" t="n"/>
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="16" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="16" t="n"/>
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="16" t="n"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="16" t="n"/>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="16" t="n"/>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="16" t="n"/>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="16" t="n"/>
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="16" t="n"/>
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="16" t="n"/>
+      <c r="C59" s="15" t="n"/>
+      <c r="D59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="16" t="n"/>
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="16" t="n"/>
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="16" t="n"/>
+      <c r="C62" s="15" t="n"/>
+      <c r="D62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="16" t="n"/>
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="16" t="n"/>
+      <c r="C64" s="15" t="n"/>
+      <c r="D64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="16" t="n"/>
+      <c r="C65" s="15" t="n"/>
+      <c r="D65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="16" t="n"/>
+      <c r="C66" s="15" t="n"/>
+      <c r="D66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="16" t="n"/>
+      <c r="C67" s="15" t="n"/>
+      <c r="D67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="16" t="n"/>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="16" t="n"/>
+      <c r="C69" s="15" t="n"/>
+      <c r="D69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="16" t="n"/>
+      <c r="C70" s="15" t="n"/>
+      <c r="D70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="16" t="n"/>
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="16" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="16" t="n"/>
+      <c r="C72" s="15" t="n"/>
+      <c r="D72" s="16" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="16" t="n"/>
+      <c r="C73" s="15" t="n"/>
+      <c r="D73" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="16" t="n"/>
+      <c r="C74" s="15" t="n"/>
+      <c r="D74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="16" t="n"/>
+      <c r="C75" s="15" t="n"/>
+      <c r="D75" s="16" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="16" t="n"/>
+      <c r="C76" s="15" t="n"/>
+      <c r="D76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="16" t="n"/>
+      <c r="C77" s="15" t="n"/>
+      <c r="D77" s="16" t="n"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="16" t="n"/>
+      <c r="C78" s="15" t="n"/>
+      <c r="D78" s="16" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rename 彈匣選擇箱 to 彈匣箱 and fix 0926 核心 record in Sheet_ori
- Rename the 層級二 item 彈匣選擇箱 (一般彈匣選擇箱 in 工作表2) to 彈匣箱
  in sheet.html, Sheet.xlsx and Sheet_ori.xlsx
- Move 0926 records 26532977040 / 18573083924 from 穩定的核心1個 to
  層級三 核心1個 in Sheet_ori.xlsx, matching sheet.html and Sheet.xlsx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -1017,7 +1017,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>一般彈匣選擇箱</t>
+          <t>彈匣箱</t>
         </is>
       </c>
       <c r="B11" s="43" t="n"/>
@@ -2416,7 +2416,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>彈匣選擇箱</t>
+          <t>彈匣箱</t>
         </is>
       </c>
       <c r="B11" s="43">
@@ -3704,7 +3704,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>彈匣選擇箱</t>
+          <t>彈匣箱</t>
         </is>
       </c>
       <c r="B11" s="43">
@@ -4971,7 +4971,7 @@
     <row r="11" ht="16.5" customHeight="1" s="10">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>彈匣選擇箱</t>
+          <t>彈匣箱</t>
         </is>
       </c>
       <c r="B11" s="43">

</xml_diff>

<commit_message>
Add imported 0930 records to sheet.html and Sheet.xlsx
- 0930 records imported via the page upload UI: 核心備份模塊3個,
  一般彈匣魔方, 每周鍛造材料1000個/2000個, 彈匣箱
- Mirror them into Sheet.xlsx 0930紀錄 and 歷史成交總集

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -2077,7 +2077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:S78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="40.5703125" customWidth="1" style="10" min="1" max="1"/>
@@ -2205,6 +2205,9 @@
       <c r="R4" t="n">
         <v>347287500</v>
       </c>
+      <c r="S4" t="n">
+        <v>942824568</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="10">
       <c r="A5" s="3" t="inlineStr">
@@ -2391,8 +2394,12 @@
       <c r="G9" s="56" t="n">
         <v>630000000</v>
       </c>
-      <c r="H9" s="56" t="n"/>
-      <c r="I9" s="56" t="n"/>
+      <c r="H9" s="56" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="I9" s="56" t="n">
+        <v>1583945273</v>
+      </c>
       <c r="J9" s="56" t="n"/>
       <c r="K9" s="56" t="n"/>
     </row>
@@ -2439,8 +2446,12 @@
       <c r="G11" s="56" t="n">
         <v>551250000</v>
       </c>
-      <c r="H11" s="56" t="n"/>
-      <c r="I11" s="56" t="n"/>
+      <c r="H11" s="56" t="n">
+        <v>551250000</v>
+      </c>
+      <c r="I11" s="56" t="n">
+        <v>3150000000</v>
+      </c>
       <c r="J11" s="56" t="n"/>
       <c r="K11" s="56" t="n"/>
     </row>
@@ -2600,8 +2611,12 @@
       <c r="E15" s="56" t="n">
         <v>136500000</v>
       </c>
-      <c r="F15" s="56" t="n"/>
-      <c r="G15" s="56" t="n"/>
+      <c r="F15" s="56" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="G15" s="56" t="n">
+        <v>36465187</v>
+      </c>
       <c r="H15" s="56" t="n"/>
       <c r="I15" s="56" t="n"/>
       <c r="J15" s="56" t="n"/>
@@ -2678,6 +2693,9 @@
         <v>400000000</v>
       </c>
       <c r="K17" s="56" t="n">
+        <v>926100000</v>
+      </c>
+      <c r="L17" t="n">
         <v>926100000</v>
       </c>
     </row>
@@ -4774,6 +4792,9 @@
       <c r="L4" t="n">
         <v>347287500</v>
       </c>
+      <c r="M4" t="n">
+        <v>942824568</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="10">
       <c r="A5" s="3" t="inlineStr">
@@ -4944,8 +4965,12 @@
       <c r="E9" s="56" t="n">
         <v>630000000</v>
       </c>
-      <c r="F9" s="56" t="n"/>
-      <c r="G9" s="56" t="n"/>
+      <c r="F9" s="56" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="G9" s="56" t="n">
+        <v>1583945273</v>
+      </c>
       <c r="H9" s="56" t="n"/>
       <c r="I9" s="56" t="n"/>
       <c r="J9" s="56" t="n"/>
@@ -4991,8 +5016,12 @@
       <c r="F11" s="56" t="n">
         <v>551250000</v>
       </c>
-      <c r="G11" s="56" t="n"/>
-      <c r="H11" s="56" t="n"/>
+      <c r="G11" s="56" t="n">
+        <v>551250000</v>
+      </c>
+      <c r="H11" s="56" t="n">
+        <v>3150000000</v>
+      </c>
       <c r="I11" s="56" t="n"/>
       <c r="J11" s="56" t="n"/>
       <c r="K11" s="56" t="n"/>
@@ -5126,8 +5155,12 @@
       <c r="E15" s="56" t="n">
         <v>136500000</v>
       </c>
-      <c r="F15" s="56" t="n"/>
-      <c r="G15" s="56" t="n"/>
+      <c r="F15" s="56" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="G15" s="56" t="n">
+        <v>36465187</v>
+      </c>
       <c r="H15" s="56" t="n"/>
       <c r="I15" s="56" t="n"/>
       <c r="J15" s="56" t="n"/>
@@ -5191,7 +5224,9 @@
       <c r="J17" s="56" t="n">
         <v>926100000</v>
       </c>
-      <c r="K17" s="56" t="n"/>
+      <c r="K17" s="56" t="n">
+        <v>926100000</v>
+      </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="10">
       <c r="A18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add 1014 records to sheet.html and Sheet.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C981901F-DBF9-4078-BFEE-F2041E45EFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6273251-1C51-4823-B187-EE585D673720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="1003紀錄" sheetId="6" r:id="rId6"/>
     <sheet name="1007紀錄" sheetId="7" r:id="rId7"/>
     <sheet name="1010紀錄" sheetId="9" r:id="rId8"/>
+    <sheet name="1014紀錄" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -315,8 +316,34 @@
 </comments>
 </file>
 
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{63F3312C-244E-4C78-9F00-2FC0BA037A22}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="60">
   <si>
     <t>Last Update: 20260914</t>
   </si>
@@ -9230,4 +9257,1185 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9C88A78-9C2A-4880-92F8-630536B2A945}">
+  <dimension ref="A1:N78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>46309</v>
+      </c>
+      <c r="E2" s="30">
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>505390030</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>2016726678</v>
+      </c>
+      <c r="D4" s="21">
+        <v>505390030</v>
+      </c>
+      <c r="E4" s="32">
+        <v>551250000</v>
+      </c>
+      <c r="F4" s="32">
+        <v>593979474</v>
+      </c>
+      <c r="G4" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="H4" s="32">
+        <v>2016726678</v>
+      </c>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+    </row>
+    <row r="5" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>124106255</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>600000000</v>
+      </c>
+      <c r="D5" s="19">
+        <v>124106255</v>
+      </c>
+      <c r="E5" s="32">
+        <v>359171262</v>
+      </c>
+      <c r="F5" s="32">
+        <v>600000000</v>
+      </c>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+    </row>
+    <row r="6" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>578812500</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>1050000000</v>
+      </c>
+      <c r="D6" s="19">
+        <v>620000000</v>
+      </c>
+      <c r="E6" s="32">
+        <v>735000000</v>
+      </c>
+      <c r="F6" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="G6" s="32">
+        <v>578812500</v>
+      </c>
+      <c r="H6" s="32">
+        <v>1050000000</v>
+      </c>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>500000000</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>500000000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>500000000</v>
+      </c>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>11025000</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>210000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>115500000</v>
+      </c>
+      <c r="E8" s="32">
+        <v>127628156</v>
+      </c>
+      <c r="F8" s="32">
+        <v>21828737</v>
+      </c>
+      <c r="G8" s="32">
+        <v>11025000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>60000000</v>
+      </c>
+      <c r="I8" s="32">
+        <v>50000000</v>
+      </c>
+      <c r="J8" s="32">
+        <v>14071002</v>
+      </c>
+      <c r="K8" s="32">
+        <v>210000000</v>
+      </c>
+      <c r="L8" s="35">
+        <v>35556707</v>
+      </c>
+      <c r="M8" s="35">
+        <v>171033934</v>
+      </c>
+      <c r="N8" s="35">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>1050000000</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>3677415513</v>
+      </c>
+      <c r="D9" s="19">
+        <v>2000000000</v>
+      </c>
+      <c r="E9" s="32">
+        <v>1050000000</v>
+      </c>
+      <c r="F9" s="32">
+        <v>3677415513</v>
+      </c>
+      <c r="G9" s="32">
+        <v>3257789252</v>
+      </c>
+      <c r="H9" s="32">
+        <v>3500000000</v>
+      </c>
+      <c r="I9" s="32">
+        <v>2110650633</v>
+      </c>
+      <c r="J9" s="32">
+        <v>1653750000</v>
+      </c>
+      <c r="K9" s="32"/>
+    </row>
+    <row r="10" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>330750000</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>3402413451</v>
+      </c>
+      <c r="D11" s="19">
+        <v>3292908451</v>
+      </c>
+      <c r="E11" s="32">
+        <v>600000000</v>
+      </c>
+      <c r="F11" s="32">
+        <v>3402413451</v>
+      </c>
+      <c r="G11" s="32">
+        <v>700000000</v>
+      </c>
+      <c r="H11" s="32">
+        <v>2925260709</v>
+      </c>
+      <c r="I11" s="32">
+        <v>1102500000</v>
+      </c>
+      <c r="J11" s="32">
+        <v>330750000</v>
+      </c>
+      <c r="K11" s="32">
+        <v>500000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>200000000</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>3095620928</v>
+      </c>
+      <c r="D12" s="19">
+        <v>1710339356</v>
+      </c>
+      <c r="E12" s="32">
+        <v>200000000</v>
+      </c>
+      <c r="F12" s="32">
+        <v>1755156420</v>
+      </c>
+      <c r="G12" s="32">
+        <v>3095620928</v>
+      </c>
+      <c r="H12" s="32">
+        <v>977336773</v>
+      </c>
+      <c r="I12" s="32">
+        <v>1257099423</v>
+      </c>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>1247356901</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1881373290</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1881373290</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1247356901</v>
+      </c>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>570113111</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>1535761867</v>
+      </c>
+      <c r="D14" s="19">
+        <v>700000000</v>
+      </c>
+      <c r="E14" s="32">
+        <v>570113111</v>
+      </c>
+      <c r="F14" s="32">
+        <v>1535761867</v>
+      </c>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>31500000</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>207892813</v>
+      </c>
+      <c r="D15" s="19">
+        <v>31500000</v>
+      </c>
+      <c r="E15" s="32">
+        <v>51310177</v>
+      </c>
+      <c r="F15" s="32">
+        <v>207892813</v>
+      </c>
+      <c r="G15" s="32">
+        <v>44323661</v>
+      </c>
+      <c r="H15" s="32">
+        <v>42213011</v>
+      </c>
+      <c r="I15" s="32">
+        <v>162889461</v>
+      </c>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+    </row>
+    <row r="16" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>3000000000</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>8144473130</v>
+      </c>
+      <c r="D17" s="19">
+        <v>3000000000</v>
+      </c>
+      <c r="E17" s="32">
+        <v>8144473130</v>
+      </c>
+      <c r="F17" s="32">
+        <v>3675000000</v>
+      </c>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>5400000000</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>5400000000</v>
+      </c>
+      <c r="D19" s="19">
+        <v>5400000000</v>
+      </c>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>14332500000</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>20101434608</v>
+      </c>
+      <c r="D20" s="19">
+        <v>14332500000</v>
+      </c>
+      <c r="E20" s="32">
+        <v>20101434608</v>
+      </c>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>7387277217</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>8682187500</v>
+      </c>
+      <c r="D21" s="19">
+        <v>7387277217</v>
+      </c>
+      <c r="E21" s="32">
+        <v>8682187500</v>
+      </c>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="19"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="19"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>700000000</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>700000000</v>
+      </c>
+      <c r="D32" s="19">
+        <v>700000000</v>
+      </c>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 1017 records to sheet.html and Sheet.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6273251-1C51-4823-B187-EE585D673720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21B2DD8-2815-4DF1-9C18-41923447F183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="1007紀錄" sheetId="7" r:id="rId7"/>
     <sheet name="1010紀錄" sheetId="9" r:id="rId8"/>
     <sheet name="1014紀錄" sheetId="10" r:id="rId9"/>
+    <sheet name="1017紀錄" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -342,8 +343,34 @@
 </comments>
 </file>
 
+<file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{202ACD26-8ED9-491C-8699-46C5B281D1DE}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="60">
   <si>
     <t>Last Update: 20260914</t>
   </si>
@@ -1921,6 +1948,1211 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{514374CC-C5DA-4317-87E2-42FF1F07BC3C}">
+  <dimension ref="A1:N78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1021</v>
+      </c>
+      <c r="E2" s="30">
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>240661916</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>2756250000</v>
+      </c>
+      <c r="D4" s="21">
+        <v>2000000000</v>
+      </c>
+      <c r="E4" s="32">
+        <v>900000000</v>
+      </c>
+      <c r="F4" s="32">
+        <v>240661916</v>
+      </c>
+      <c r="G4" s="32">
+        <v>2756250000</v>
+      </c>
+      <c r="H4" s="32">
+        <v>2309461875</v>
+      </c>
+      <c r="I4" s="32">
+        <v>1000000000</v>
+      </c>
+      <c r="J4" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="K4" s="32">
+        <v>2431012500</v>
+      </c>
+      <c r="L4" s="35">
+        <v>1000000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>492485146</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>492485146</v>
+      </c>
+      <c r="D5" s="19">
+        <v>492485146</v>
+      </c>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+    </row>
+    <row r="6" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>720000000</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>930796927</v>
+      </c>
+      <c r="D6" s="19">
+        <v>844260252</v>
+      </c>
+      <c r="E6" s="32">
+        <v>720000000</v>
+      </c>
+      <c r="F6" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="G6" s="32">
+        <v>930796927</v>
+      </c>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>100000000</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>525000000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>210000000</v>
+      </c>
+      <c r="E7" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>310265641</v>
+      </c>
+      <c r="G7" s="32">
+        <v>200000000</v>
+      </c>
+      <c r="H7" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="I7" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="J7" s="32">
+        <v>105000000</v>
+      </c>
+      <c r="K7" s="32">
+        <v>240661916</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>13400955</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>300000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>300000000</v>
+      </c>
+      <c r="E8" s="32">
+        <v>200000000</v>
+      </c>
+      <c r="F8" s="32">
+        <v>13400955</v>
+      </c>
+      <c r="G8" s="32">
+        <v>40000000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>50000000</v>
+      </c>
+      <c r="I8" s="32">
+        <v>42213011</v>
+      </c>
+      <c r="J8" s="32">
+        <v>110250000</v>
+      </c>
+      <c r="K8" s="32">
+        <v>52533446</v>
+      </c>
+      <c r="L8" s="35">
+        <v>17958558</v>
+      </c>
+      <c r="M8" s="35">
+        <v>115762500</v>
+      </c>
+      <c r="N8" s="35"/>
+    </row>
+    <row r="9" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>2110650633</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>2680191281</v>
+      </c>
+      <c r="D9" s="19">
+        <v>2680191281</v>
+      </c>
+      <c r="E9" s="32">
+        <v>2110650633</v>
+      </c>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+    </row>
+    <row r="10" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>1260000000</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>3307500000</v>
+      </c>
+      <c r="D11" s="19">
+        <v>2000000000</v>
+      </c>
+      <c r="E11" s="32">
+        <v>2500000000</v>
+      </c>
+      <c r="F11" s="32">
+        <v>3307500000</v>
+      </c>
+      <c r="G11" s="32">
+        <v>1260000000</v>
+      </c>
+      <c r="H11" s="32">
+        <v>1888888888</v>
+      </c>
+      <c r="I11" s="32">
+        <v>2117563011</v>
+      </c>
+      <c r="J11" s="32">
+        <v>2406619226</v>
+      </c>
+      <c r="K11" s="32">
+        <v>1551328215</v>
+      </c>
+      <c r="L11" s="35">
+        <v>2500000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>1010780070</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>5512500000</v>
+      </c>
+      <c r="D12" s="19">
+        <v>5512500000</v>
+      </c>
+      <c r="E12" s="32">
+        <v>1281000000</v>
+      </c>
+      <c r="F12" s="32">
+        <v>1500000000</v>
+      </c>
+      <c r="G12" s="32">
+        <v>1041596666</v>
+      </c>
+      <c r="H12" s="32">
+        <v>1010780070</v>
+      </c>
+      <c r="I12" s="32">
+        <v>3646518750</v>
+      </c>
+      <c r="J12" s="32">
+        <v>1385952113</v>
+      </c>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>525000000</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1500000000</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1050000000</v>
+      </c>
+      <c r="E13" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="F13" s="32">
+        <v>1500000000</v>
+      </c>
+      <c r="G13" s="32">
+        <v>1286249997</v>
+      </c>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>150000000</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>989965796</v>
+      </c>
+      <c r="D14" s="19">
+        <v>638140781</v>
+      </c>
+      <c r="E14" s="32">
+        <v>150000000</v>
+      </c>
+      <c r="F14" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="G14" s="32">
+        <v>218882282</v>
+      </c>
+      <c r="H14" s="32">
+        <v>989965796</v>
+      </c>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>33075000</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>315000000</v>
+      </c>
+      <c r="D15" s="19">
+        <v>315000000</v>
+      </c>
+      <c r="E15" s="32">
+        <v>68760541</v>
+      </c>
+      <c r="F15" s="32">
+        <v>33075000</v>
+      </c>
+      <c r="G15" s="32">
+        <v>63814077</v>
+      </c>
+      <c r="H15" s="32">
+        <v>142948218</v>
+      </c>
+      <c r="I15" s="32">
+        <v>140710041</v>
+      </c>
+      <c r="J15" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="K15" s="32">
+        <v>110250000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>3038765625</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>8551696786</v>
+      </c>
+      <c r="D17" s="19">
+        <v>6548623758</v>
+      </c>
+      <c r="E17" s="32">
+        <v>8551696786</v>
+      </c>
+      <c r="F17" s="32">
+        <v>6077531250</v>
+      </c>
+      <c r="G17" s="32">
+        <v>3038765625</v>
+      </c>
+      <c r="H17" s="32">
+        <v>3693638608</v>
+      </c>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>3150000000</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>5250000000</v>
+      </c>
+      <c r="D23" s="19">
+        <v>3150000000</v>
+      </c>
+      <c r="E23" s="32">
+        <v>5250000000</v>
+      </c>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>897928160</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>897928160</v>
+      </c>
+      <c r="D24" s="19">
+        <v>897928160</v>
+      </c>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>200000000</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>200000000</v>
+      </c>
+      <c r="D25" s="19">
+        <v>200000000</v>
+      </c>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>24310125000</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>24310125000</v>
+      </c>
+      <c r="D36" s="19">
+        <v>24310125000</v>
+      </c>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:B41"/>

</xml_diff>

<commit_message>
Fix 1014 核心1個 record: 5400000000 -> 8400000000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21B2DD8-2815-4DF1-9C18-41923447F183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAB0B148-5E0D-4A39-BBD5-B94A20BCEB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -10994,14 +10994,14 @@
       </c>
       <c r="B19" s="19">
         <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
-        <v>5400000000</v>
+        <v>8400000000</v>
       </c>
       <c r="C19" s="20">
         <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
-        <v>5400000000</v>
+        <v>8400000000</v>
       </c>
       <c r="D19" s="19">
-        <v>5400000000</v>
+        <v>8400000000</v>
       </c>
       <c r="E19" s="32"/>
       <c r="F19" s="32"/>

</xml_diff>

<commit_message>
Add 1021 records to sheet.html and Sheet.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAB0B148-5E0D-4A39-BBD5-B94A20BCEB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB250DC6-5802-455F-9729-038C9EF82747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="1010紀錄" sheetId="9" r:id="rId8"/>
     <sheet name="1014紀錄" sheetId="10" r:id="rId9"/>
     <sheet name="1017紀錄" sheetId="11" r:id="rId10"/>
+    <sheet name="1021紀錄" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -154,6 +155,32 @@
           </rPr>
           <t>USER:
 先當40個黑色碎片</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{33381E55-2345-457E-80F3-C44652603E66}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
         </r>
       </text>
     </comment>
@@ -370,7 +397,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="60">
   <si>
     <t>Last Update: 20260914</t>
   </si>
@@ -3153,6 +3180,1151 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E06DFE8-572C-459B-99C6-75CE6A4CBB59}">
+  <dimension ref="A1:N78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1025</v>
+      </c>
+      <c r="E2" s="30">
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>1905976563</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>1905976563</v>
+      </c>
+      <c r="D4" s="21">
+        <v>1905976563</v>
+      </c>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="35"/>
+    </row>
+    <row r="5" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>300000000</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>525334771</v>
+      </c>
+      <c r="D5" s="19">
+        <v>300000000</v>
+      </c>
+      <c r="E5" s="32">
+        <v>343802737</v>
+      </c>
+      <c r="F5" s="32">
+        <v>525334771</v>
+      </c>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+    </row>
+    <row r="6" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>422130125</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>900000000</v>
+      </c>
+      <c r="D6" s="19">
+        <v>687605487</v>
+      </c>
+      <c r="E6" s="32">
+        <v>900000000</v>
+      </c>
+      <c r="F6" s="32">
+        <v>422130125</v>
+      </c>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>17103389</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>992250000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>17103389</v>
+      </c>
+      <c r="E7" s="32">
+        <v>300000000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>35177508</v>
+      </c>
+      <c r="G7" s="32">
+        <v>992250000</v>
+      </c>
+      <c r="H7" s="32">
+        <v>565694738</v>
+      </c>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>30000000</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>105000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>100000000</v>
+      </c>
+      <c r="E8" s="32">
+        <v>67004780</v>
+      </c>
+      <c r="F8" s="32">
+        <v>30000000</v>
+      </c>
+      <c r="G8" s="32">
+        <v>80000000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>84000000</v>
+      </c>
+      <c r="I8" s="32">
+        <v>105000000</v>
+      </c>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="35"/>
+      <c r="M8" s="35"/>
+      <c r="N8" s="35"/>
+    </row>
+    <row r="9" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>1102500000</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>4020286921</v>
+      </c>
+      <c r="D9" s="19">
+        <v>1157625000</v>
+      </c>
+      <c r="E9" s="32">
+        <v>1102500000</v>
+      </c>
+      <c r="F9" s="32">
+        <v>4020286921</v>
+      </c>
+      <c r="G9" s="32">
+        <v>3141011917</v>
+      </c>
+      <c r="H9" s="32">
+        <v>2979623803</v>
+      </c>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+    </row>
+    <row r="10" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>3828844687</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>3828844687</v>
+      </c>
+      <c r="D11" s="19">
+        <v>3828844687</v>
+      </c>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="35"/>
+    </row>
+    <row r="12" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>1146009153</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>1979931595</v>
+      </c>
+      <c r="D12" s="19">
+        <v>1979931595</v>
+      </c>
+      <c r="E12" s="32">
+        <v>1146009153</v>
+      </c>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>1329709897</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1608114768</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1329709897</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1458607500</v>
+      </c>
+      <c r="F13" s="32">
+        <v>1608114768</v>
+      </c>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>500000000</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>1303115698</v>
+      </c>
+      <c r="D14" s="19">
+        <v>500000000</v>
+      </c>
+      <c r="E14" s="32">
+        <v>1303115698</v>
+      </c>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>100000000</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>300000000</v>
+      </c>
+      <c r="D15" s="19">
+        <v>150000000</v>
+      </c>
+      <c r="E15" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="F15" s="32">
+        <v>300000000</v>
+      </c>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+    </row>
+    <row r="16" spans="1:14" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>2292018311</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>4886683878</v>
+      </c>
+      <c r="D17" s="19">
+        <v>2292018311</v>
+      </c>
+      <c r="E17" s="32">
+        <v>3790425284</v>
+      </c>
+      <c r="F17" s="32">
+        <v>4886683878</v>
+      </c>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>10500000000</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>20000000000</v>
+      </c>
+      <c r="D19" s="19">
+        <v>10500000000</v>
+      </c>
+      <c r="E19" s="32">
+        <v>20000000000</v>
+      </c>
+      <c r="F19" s="32">
+        <v>19799315988</v>
+      </c>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>19799315988</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>19799315988</v>
+      </c>
+      <c r="D20" s="19">
+        <v>19799315988</v>
+      </c>
+      <c r="E20" s="32">
+        <v>19799315988</v>
+      </c>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>20114253419</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>20114253419</v>
+      </c>
+      <c r="D21" s="19">
+        <v>20114253419</v>
+      </c>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>2626673960</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>2626673960</v>
+      </c>
+      <c r="D22" s="19">
+        <v>2626673960</v>
+      </c>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>1021025250</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>1021025250</v>
+      </c>
+      <c r="D24" s="19">
+        <v>1021025250</v>
+      </c>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>5105126250</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>5105126250</v>
+      </c>
+      <c r="D25" s="19">
+        <v>5105126250</v>
+      </c>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>10000000000</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>10000000000</v>
+      </c>
+      <c r="D27" s="19">
+        <v>10000000000</v>
+      </c>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:B41"/>

</xml_diff>

<commit_message>
Add 1024 records to sheet.html and Sheet.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB250DC6-5802-455F-9729-038C9EF82747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741A7CD8-9ECB-4FF0-B26C-02878106493D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="1014紀錄" sheetId="10" r:id="rId9"/>
     <sheet name="1017紀錄" sheetId="11" r:id="rId10"/>
     <sheet name="1021紀錄" sheetId="12" r:id="rId11"/>
+    <sheet name="1024紀錄" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -169,6 +170,32 @@
   </authors>
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0" xr:uid="{33381E55-2345-457E-80F3-C44652603E66}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{C9156D68-C1B6-494D-B2E2-734972E5D8F5}">
       <text>
         <r>
           <rPr>
@@ -397,7 +424,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="60">
   <si>
     <t>Last Update: 20260914</t>
   </si>
@@ -4325,6 +4352,1238 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5587BD36-BB1C-4920-8236-6A0D8F092169}">
+  <dimension ref="A1:P78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="14" width="18.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1028</v>
+      </c>
+      <c r="E2" s="30">
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>405168750</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>5909821774</v>
+      </c>
+      <c r="D4" s="21">
+        <v>1000000000</v>
+      </c>
+      <c r="E4" s="32">
+        <v>600000000</v>
+      </c>
+      <c r="F4" s="32">
+        <v>588000000</v>
+      </c>
+      <c r="G4" s="32">
+        <v>5909821774</v>
+      </c>
+      <c r="H4" s="32">
+        <v>5250000000</v>
+      </c>
+      <c r="I4" s="32">
+        <v>405168750</v>
+      </c>
+      <c r="J4" s="32">
+        <v>486202500</v>
+      </c>
+      <c r="K4" s="32"/>
+      <c r="L4" s="35"/>
+    </row>
+    <row r="5" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>244334190</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>2163232741</v>
+      </c>
+      <c r="D5" s="19">
+        <v>600000000</v>
+      </c>
+      <c r="E5" s="32">
+        <v>500000000</v>
+      </c>
+      <c r="F5" s="32">
+        <v>244334190</v>
+      </c>
+      <c r="G5" s="32">
+        <v>738727721</v>
+      </c>
+      <c r="H5" s="32">
+        <v>1050000000</v>
+      </c>
+      <c r="I5" s="32">
+        <v>2110650633</v>
+      </c>
+      <c r="J5" s="32">
+        <v>2163232741</v>
+      </c>
+      <c r="K5" s="32">
+        <v>738727721</v>
+      </c>
+      <c r="L5" s="35">
+        <v>442231560</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>312038019</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>900000000</v>
+      </c>
+      <c r="D6" s="19">
+        <v>630000000</v>
+      </c>
+      <c r="E6" s="32">
+        <v>729303750</v>
+      </c>
+      <c r="F6" s="32">
+        <v>900000000</v>
+      </c>
+      <c r="G6" s="32">
+        <v>888888888</v>
+      </c>
+      <c r="H6" s="32">
+        <v>729303750</v>
+      </c>
+      <c r="I6" s="32">
+        <v>775664107</v>
+      </c>
+      <c r="J6" s="32">
+        <v>312038019</v>
+      </c>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>210000000</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>1102500000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>210000000</v>
+      </c>
+      <c r="E7" s="32">
+        <v>1102500000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="G7" s="32">
+        <v>357000000</v>
+      </c>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>10000000</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>200000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>11025000</v>
+      </c>
+      <c r="E8" s="32">
+        <v>200000000</v>
+      </c>
+      <c r="F8" s="32">
+        <v>21000000</v>
+      </c>
+      <c r="G8" s="32">
+        <v>21000000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>17364375</v>
+      </c>
+      <c r="I8" s="32">
+        <v>115762500</v>
+      </c>
+      <c r="J8" s="32">
+        <v>121550625</v>
+      </c>
+      <c r="K8" s="32">
+        <v>51310177</v>
+      </c>
+      <c r="L8" s="35">
+        <v>10500000</v>
+      </c>
+      <c r="M8" s="35">
+        <v>21000000</v>
+      </c>
+      <c r="N8" s="35">
+        <v>15513279</v>
+      </c>
+      <c r="O8" s="35">
+        <v>10000000</v>
+      </c>
+      <c r="P8" s="35">
+        <v>33600000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>1047375000</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>6515578505</v>
+      </c>
+      <c r="D9" s="19">
+        <v>1102500000</v>
+      </c>
+      <c r="E9" s="32">
+        <v>5131018071</v>
+      </c>
+      <c r="F9" s="32">
+        <v>1047375000</v>
+      </c>
+      <c r="G9" s="32">
+        <v>2954910887</v>
+      </c>
+      <c r="H9" s="32">
+        <v>3591712649</v>
+      </c>
+      <c r="I9" s="32">
+        <v>3017038624</v>
+      </c>
+      <c r="J9" s="32">
+        <v>3009825000</v>
+      </c>
+      <c r="K9" s="32">
+        <v>2292018311</v>
+      </c>
+      <c r="L9" s="35">
+        <v>6515578505</v>
+      </c>
+      <c r="M9" s="35">
+        <v>1319954394</v>
+      </c>
+      <c r="N9" s="35">
+        <v>1485618747</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>1000000000</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>10394640890</v>
+      </c>
+      <c r="D11" s="19">
+        <v>1964587121</v>
+      </c>
+      <c r="E11" s="32">
+        <v>1021025250</v>
+      </c>
+      <c r="F11" s="32">
+        <v>1000000000</v>
+      </c>
+      <c r="G11" s="32">
+        <v>10394640890</v>
+      </c>
+      <c r="H11" s="32">
+        <v>1653750000</v>
+      </c>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="35"/>
+    </row>
+    <row r="12" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>661500000</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>4886683878</v>
+      </c>
+      <c r="D12" s="19">
+        <v>4886683878</v>
+      </c>
+      <c r="E12" s="32">
+        <v>2271394378</v>
+      </c>
+      <c r="F12" s="32">
+        <v>661500000</v>
+      </c>
+      <c r="G12" s="32">
+        <v>2000000000</v>
+      </c>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>1100000000</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1500000000</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1500000000</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1100000000</v>
+      </c>
+      <c r="F13" s="32">
+        <v>1206086076</v>
+      </c>
+      <c r="G13" s="32">
+        <v>1407100422</v>
+      </c>
+      <c r="H13" s="32">
+        <v>1260000000</v>
+      </c>
+      <c r="I13" s="32">
+        <v>1204076907</v>
+      </c>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>507953220</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>2001275391</v>
+      </c>
+      <c r="D14" s="19">
+        <v>600000000</v>
+      </c>
+      <c r="E14" s="32">
+        <v>2001275391</v>
+      </c>
+      <c r="F14" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="G14" s="32">
+        <v>1015906467</v>
+      </c>
+      <c r="H14" s="32">
+        <v>507953220</v>
+      </c>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>40000000</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>338635481</v>
+      </c>
+      <c r="D15" s="19">
+        <v>70355019</v>
+      </c>
+      <c r="E15" s="32">
+        <v>93079690</v>
+      </c>
+      <c r="F15" s="32">
+        <v>55125000</v>
+      </c>
+      <c r="G15" s="32">
+        <v>262500000</v>
+      </c>
+      <c r="H15" s="32">
+        <v>134009563</v>
+      </c>
+      <c r="I15" s="32">
+        <v>338635481</v>
+      </c>
+      <c r="J15" s="32">
+        <v>40000000</v>
+      </c>
+      <c r="K15" s="32">
+        <v>115762500</v>
+      </c>
+      <c r="L15" s="35">
+        <v>261341919</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>2552563125</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>10331803125</v>
+      </c>
+      <c r="D17" s="19">
+        <v>10331803125</v>
+      </c>
+      <c r="E17" s="32">
+        <v>5000000000</v>
+      </c>
+      <c r="F17" s="32">
+        <v>5496981676</v>
+      </c>
+      <c r="G17" s="32">
+        <v>2552563125</v>
+      </c>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>22000000000</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>22000000000</v>
+      </c>
+      <c r="D20" s="19">
+        <v>22000000000</v>
+      </c>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>3063075750</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>12222222220</v>
+      </c>
+      <c r="D23" s="19">
+        <v>12222222220</v>
+      </c>
+      <c r="E23" s="32">
+        <v>3063075750</v>
+      </c>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="19"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="19"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:B41"/>

</xml_diff>

<commit_message>
Add 1028 and 1031 records to sheet.html and Sheet.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sheet.xlsx
+++ b/Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ElswordInfo\DarkElfMarket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741A7CD8-9ECB-4FF0-B26C-02878106493D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC53F4DB-1DEF-4CD2-8742-B1C145F2E202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表2" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,8 @@
     <sheet name="1017紀錄" sheetId="11" r:id="rId10"/>
     <sheet name="1021紀錄" sheetId="12" r:id="rId11"/>
     <sheet name="1024紀錄" sheetId="13" r:id="rId12"/>
+    <sheet name="1028紀錄" sheetId="14" r:id="rId13"/>
+    <sheet name="1031紀錄" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -196,6 +198,58 @@
   </authors>
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0" xr:uid="{C9156D68-C1B6-494D-B2E2-734972E5D8F5}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{94375CDC-56CC-43F7-8E92-DF77383024A5}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="新細明體"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>USER:
+假設一件成裝140 7000NT
+黑色碎片換算台幣50</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>USER</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{6E9CF76F-BE6D-48B6-82F5-A9320C711C5B}">
       <text>
         <r>
           <rPr>
@@ -424,7 +478,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="60">
   <si>
     <t>Last Update: 20260914</t>
   </si>
@@ -5584,6 +5638,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA582D04-CD14-41DC-8A95-F4D4FC9C1353}">
+  <dimension ref="A1:P78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="14" width="18.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1032</v>
+      </c>
+      <c r="E2" s="30">
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>1000000000</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>4051687500</v>
+      </c>
+      <c r="D4" s="21">
+        <v>1028999997</v>
+      </c>
+      <c r="E4" s="32">
+        <v>1000000000</v>
+      </c>
+      <c r="F4" s="32">
+        <v>4051687500</v>
+      </c>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="35"/>
+    </row>
+    <row r="5" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>420000000</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>840000000</v>
+      </c>
+      <c r="D5" s="19">
+        <v>420000000</v>
+      </c>
+      <c r="E5" s="32">
+        <v>500000000</v>
+      </c>
+      <c r="F5" s="32">
+        <v>513101804</v>
+      </c>
+      <c r="G5" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="H5" s="32">
+        <v>840000000</v>
+      </c>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="35"/>
+    </row>
+    <row r="6" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>600000000</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>945000000</v>
+      </c>
+      <c r="D6" s="19">
+        <v>600000000</v>
+      </c>
+      <c r="E6" s="32">
+        <v>893397093</v>
+      </c>
+      <c r="F6" s="32">
+        <v>721985761</v>
+      </c>
+      <c r="G6" s="32">
+        <v>945000000</v>
+      </c>
+      <c r="H6" s="32">
+        <v>775664107</v>
+      </c>
+      <c r="I6" s="32">
+        <v>840000000</v>
+      </c>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>51051262</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>500000000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>63814077</v>
+      </c>
+      <c r="E7" s="32">
+        <v>92610000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>500000000</v>
+      </c>
+      <c r="G7" s="32">
+        <v>330750000</v>
+      </c>
+      <c r="H7" s="32">
+        <v>210000000</v>
+      </c>
+      <c r="I7" s="32">
+        <v>51051262</v>
+      </c>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>10500000</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>100000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>12762815</v>
+      </c>
+      <c r="E8" s="32">
+        <v>12762815</v>
+      </c>
+      <c r="F8" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="G8" s="32">
+        <v>100000000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>22050000</v>
+      </c>
+      <c r="I8" s="32">
+        <v>10500000</v>
+      </c>
+      <c r="J8" s="32">
+        <v>14774552</v>
+      </c>
+      <c r="K8" s="32">
+        <v>40000000</v>
+      </c>
+      <c r="L8" s="35">
+        <v>63814077</v>
+      </c>
+      <c r="N8" s="35"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="35"/>
+    </row>
+    <row r="9" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>2100000000</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>2457218989</v>
+      </c>
+      <c r="D9" s="19">
+        <v>2457218989</v>
+      </c>
+      <c r="E9" s="32">
+        <v>2100000000</v>
+      </c>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+    </row>
+    <row r="10" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>1000000000</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>10500000000</v>
+      </c>
+      <c r="D11" s="19">
+        <v>10500000000</v>
+      </c>
+      <c r="E11" s="32">
+        <v>7500000000</v>
+      </c>
+      <c r="F11" s="32">
+        <v>1148653406</v>
+      </c>
+      <c r="G11" s="32">
+        <v>1000000000</v>
+      </c>
+      <c r="H11" s="32">
+        <v>1914422343</v>
+      </c>
+      <c r="I11" s="32">
+        <v>2406619226</v>
+      </c>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="35"/>
+    </row>
+    <row r="12" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>1000000000</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>1746299662</v>
+      </c>
+      <c r="D12" s="19">
+        <v>1000000000</v>
+      </c>
+      <c r="E12" s="32">
+        <v>1050000000</v>
+      </c>
+      <c r="F12" s="32">
+        <v>1093955625</v>
+      </c>
+      <c r="G12" s="32">
+        <v>1247356901</v>
+      </c>
+      <c r="H12" s="32">
+        <v>1000000000</v>
+      </c>
+      <c r="I12" s="32">
+        <v>1746299662</v>
+      </c>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>1000000000</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1407100422</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1000000000</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1407100422</v>
+      </c>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>200000000</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>315000000</v>
+      </c>
+      <c r="D14" s="19">
+        <v>200000000</v>
+      </c>
+      <c r="E14" s="32">
+        <v>315000000</v>
+      </c>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>56000000</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>178500000</v>
+      </c>
+      <c r="D15" s="19">
+        <v>56000000</v>
+      </c>
+      <c r="E15" s="32">
+        <v>127628156</v>
+      </c>
+      <c r="F15" s="32">
+        <v>121550625</v>
+      </c>
+      <c r="G15" s="32">
+        <v>105000000</v>
+      </c>
+      <c r="H15" s="32">
+        <v>178500000</v>
+      </c>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="35"/>
+    </row>
+    <row r="16" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>2756250000</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>8442602535</v>
+      </c>
+      <c r="D17" s="19">
+        <v>3307500000</v>
+      </c>
+      <c r="E17" s="32">
+        <v>2756250000</v>
+      </c>
+      <c r="F17" s="32">
+        <v>5105126250</v>
+      </c>
+      <c r="G17" s="32">
+        <v>5131018071</v>
+      </c>
+      <c r="H17" s="32">
+        <v>8442602535</v>
+      </c>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>14774554437</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>14774554437</v>
+      </c>
+      <c r="D19" s="19">
+        <v>14774554437</v>
+      </c>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>24121721531</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>24121721531</v>
+      </c>
+      <c r="D20" s="19">
+        <v>24121721531</v>
+      </c>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>2000000000</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>2785962580</v>
+      </c>
+      <c r="D22" s="19">
+        <v>2000000000</v>
+      </c>
+      <c r="E22" s="32">
+        <v>2785962580</v>
+      </c>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="19"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>565694738</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>565694738</v>
+      </c>
+      <c r="D25" s="19">
+        <v>565694738</v>
+      </c>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE1BCD61-E118-4910-9D54-E4A26838EF33}">
+  <dimension ref="A1:P78"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="40.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="7" customWidth="1"/>
+    <col min="7" max="8" width="18.28515625" style="16" customWidth="1"/>
+    <col min="9" max="10" width="18.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="14" width="18.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="29">
+        <v>1035</v>
+      </c>
+      <c r="E2" s="30">
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B9" si="0">MIN(D4:AZ4)</f>
+        <v>538756894</v>
+      </c>
+      <c r="C4" s="20">
+        <f t="shared" ref="C4:C9" si="1">MAX(D4:AZ4)</f>
+        <v>3150000000</v>
+      </c>
+      <c r="D4" s="21">
+        <v>718182853</v>
+      </c>
+      <c r="E4" s="32">
+        <v>538756894</v>
+      </c>
+      <c r="F4" s="32">
+        <v>3150000000</v>
+      </c>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="35"/>
+    </row>
+    <row r="5" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>443236631</v>
+      </c>
+      <c r="C5" s="20">
+        <f t="shared" si="1"/>
+        <v>1187958954</v>
+      </c>
+      <c r="D5" s="19">
+        <v>1021025250</v>
+      </c>
+      <c r="E5" s="32">
+        <v>443236631</v>
+      </c>
+      <c r="F5" s="32">
+        <v>1187958954</v>
+      </c>
+      <c r="G5" s="32">
+        <v>525000000</v>
+      </c>
+      <c r="H5" s="32">
+        <v>500000000</v>
+      </c>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="35"/>
+    </row>
+    <row r="6" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>840000000</v>
+      </c>
+      <c r="C6" s="20">
+        <f t="shared" si="1"/>
+        <v>926100000</v>
+      </c>
+      <c r="D6" s="19">
+        <v>926100000</v>
+      </c>
+      <c r="E6" s="32">
+        <v>855169677</v>
+      </c>
+      <c r="F6" s="32">
+        <v>882000000</v>
+      </c>
+      <c r="G6" s="32">
+        <v>840000000</v>
+      </c>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="19">
+        <f>MIN(D7:AZ7)</f>
+        <v>173643750</v>
+      </c>
+      <c r="C7" s="20">
+        <f>MAX(D7:AZ7)</f>
+        <v>1500000000</v>
+      </c>
+      <c r="D7" s="19">
+        <v>182325937</v>
+      </c>
+      <c r="E7" s="32">
+        <v>1500000000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>347287500</v>
+      </c>
+      <c r="G7" s="32">
+        <v>200000000</v>
+      </c>
+      <c r="H7" s="32">
+        <v>173643750</v>
+      </c>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>10000000</v>
+      </c>
+      <c r="C8" s="20">
+        <f t="shared" si="1"/>
+        <v>100000000</v>
+      </c>
+      <c r="D8" s="19">
+        <v>100000000</v>
+      </c>
+      <c r="E8" s="32">
+        <v>70000000</v>
+      </c>
+      <c r="F8" s="32">
+        <v>31500000</v>
+      </c>
+      <c r="G8" s="32">
+        <v>10000000</v>
+      </c>
+      <c r="H8" s="32">
+        <v>11576250</v>
+      </c>
+      <c r="I8" s="32">
+        <v>12762815</v>
+      </c>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="35"/>
+      <c r="M8" s="35"/>
+      <c r="N8" s="35"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="35"/>
+    </row>
+    <row r="9" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>2010143460</v>
+      </c>
+      <c r="C9" s="20">
+        <f t="shared" si="1"/>
+        <v>6236784532</v>
+      </c>
+      <c r="D9" s="19">
+        <v>2954910887</v>
+      </c>
+      <c r="E9" s="32">
+        <v>4410000000</v>
+      </c>
+      <c r="F9" s="32">
+        <v>5512500000</v>
+      </c>
+      <c r="G9" s="32">
+        <v>2110650633</v>
+      </c>
+      <c r="H9" s="32">
+        <v>2010143460</v>
+      </c>
+      <c r="I9" s="32">
+        <v>6236784532</v>
+      </c>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+    </row>
+    <row r="10" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+    </row>
+    <row r="11" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="19">
+        <f t="shared" ref="B11:B17" si="2">MIN(D11:AZ11)</f>
+        <v>800000000</v>
+      </c>
+      <c r="C11" s="20">
+        <f t="shared" ref="C11:C17" si="3">MAX(D11:AZ11)</f>
+        <v>7875000000</v>
+      </c>
+      <c r="D11" s="19">
+        <v>1000000000</v>
+      </c>
+      <c r="E11" s="32">
+        <v>800000000</v>
+      </c>
+      <c r="F11" s="32">
+        <v>1407100422</v>
+      </c>
+      <c r="G11" s="32">
+        <v>7875000000</v>
+      </c>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="35"/>
+    </row>
+    <row r="12" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="19">
+        <f t="shared" si="2"/>
+        <v>670047820</v>
+      </c>
+      <c r="C12" s="20">
+        <f t="shared" si="3"/>
+        <v>1290039964</v>
+      </c>
+      <c r="D12" s="19">
+        <v>1290039964</v>
+      </c>
+      <c r="E12" s="32">
+        <v>989965796</v>
+      </c>
+      <c r="F12" s="32">
+        <v>670047820</v>
+      </c>
+      <c r="G12" s="32">
+        <v>1146009153</v>
+      </c>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="19">
+        <f t="shared" si="2"/>
+        <v>1000000000</v>
+      </c>
+      <c r="C13" s="20">
+        <f t="shared" si="3"/>
+        <v>1653750000</v>
+      </c>
+      <c r="D13" s="19">
+        <v>1000000000</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1365000000</v>
+      </c>
+      <c r="F13" s="32">
+        <v>1433250000</v>
+      </c>
+      <c r="G13" s="32">
+        <v>1653750000</v>
+      </c>
+      <c r="H13" s="32">
+        <v>1500000000</v>
+      </c>
+      <c r="I13" s="32">
+        <v>1263475090</v>
+      </c>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19">
+        <f t="shared" si="2"/>
+        <v>513101804</v>
+      </c>
+      <c r="C14" s="20">
+        <f t="shared" si="3"/>
+        <v>1981194156</v>
+      </c>
+      <c r="D14" s="19">
+        <v>800000000</v>
+      </c>
+      <c r="E14" s="32">
+        <v>661500000</v>
+      </c>
+      <c r="F14" s="32">
+        <v>703550211</v>
+      </c>
+      <c r="G14" s="32">
+        <v>1981194156</v>
+      </c>
+      <c r="H14" s="32">
+        <v>804057383</v>
+      </c>
+      <c r="I14" s="32">
+        <v>630000000</v>
+      </c>
+      <c r="J14" s="32">
+        <v>513101804</v>
+      </c>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="19">
+        <f t="shared" si="2"/>
+        <v>40202868</v>
+      </c>
+      <c r="C15" s="20">
+        <f t="shared" si="3"/>
+        <v>420000000</v>
+      </c>
+      <c r="D15" s="19">
+        <v>191442233</v>
+      </c>
+      <c r="E15" s="32">
+        <v>420000000</v>
+      </c>
+      <c r="F15" s="32">
+        <v>110250000</v>
+      </c>
+      <c r="G15" s="32">
+        <v>40202868</v>
+      </c>
+      <c r="H15" s="32">
+        <v>101590632</v>
+      </c>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="35"/>
+    </row>
+    <row r="16" spans="1:16" ht="16.5" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="19">
+        <f t="shared" si="2"/>
+        <v>3675000000</v>
+      </c>
+      <c r="C17" s="20">
+        <f t="shared" si="3"/>
+        <v>3675000000</v>
+      </c>
+      <c r="D17" s="19">
+        <v>3675000000</v>
+      </c>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
+        <f t="shared" ref="B19:B25" si="4">MIN(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <f t="shared" ref="C19:C25" si="5">MAX(D19:AZ19)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C20" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="19">
+        <f t="shared" si="4"/>
+        <v>7387277217</v>
+      </c>
+      <c r="C21" s="20">
+        <f t="shared" si="5"/>
+        <v>10939556250</v>
+      </c>
+      <c r="D21" s="19">
+        <v>7919726394</v>
+      </c>
+      <c r="E21" s="32">
+        <v>7387277217</v>
+      </c>
+      <c r="F21" s="32">
+        <v>10939556250</v>
+      </c>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C23" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="19">
+        <f t="shared" si="4"/>
+        <v>105000000</v>
+      </c>
+      <c r="C24" s="20">
+        <f t="shared" si="5"/>
+        <v>105000000</v>
+      </c>
+      <c r="D24" s="19">
+        <v>105000000</v>
+      </c>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="C25" s="20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="19"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="19">
+        <f t="shared" ref="B27:B34" si="6">MIN(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="20">
+        <f t="shared" ref="C27:C34" si="7">MAX(D27:AZ27)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C30" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A31" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="19">
+        <f t="shared" si="6"/>
+        <v>7542596566</v>
+      </c>
+      <c r="C31" s="20">
+        <f t="shared" si="7"/>
+        <v>7542596566</v>
+      </c>
+      <c r="D31" s="19">
+        <v>7542596566</v>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="19">
+        <f t="shared" si="6"/>
+        <v>165375000</v>
+      </c>
+      <c r="C32" s="20">
+        <f t="shared" si="7"/>
+        <v>165375000</v>
+      </c>
+      <c r="D32" s="19">
+        <v>165375000</v>
+      </c>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="19">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="C33" s="20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="19">
+        <f t="shared" si="6"/>
+        <v>500000000</v>
+      </c>
+      <c r="C34" s="20">
+        <f t="shared" si="7"/>
+        <v>500000000</v>
+      </c>
+      <c r="D34" s="19">
+        <v>500000000</v>
+      </c>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="19">
+        <f t="shared" ref="B36:B41" si="8">MIN(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="20">
+        <f t="shared" ref="C36:C41" si="9">MAX(D36:AZ36)</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+    </row>
+    <row r="37" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D37" s="19"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
+      <c r="K37" s="32"/>
+    </row>
+    <row r="38" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D38" s="19"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+    </row>
+    <row r="39" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+    </row>
+    <row r="40" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+    </row>
+    <row r="41" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="20">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+    </row>
+    <row r="42" spans="1:11" ht="16.5" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="B44" s="12"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="B47" s="12"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="2:4">
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="2:4">
+      <c r="B50" s="12"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="2:4">
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="2:4">
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="2:4">
+      <c r="B53" s="12"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="2:4">
+      <c r="B54" s="12"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="2:4">
+      <c r="B55" s="12"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="2:4">
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="12"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="12"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="2:4">
+      <c r="B59" s="12"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="2:4">
+      <c r="B60" s="12"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
+    </row>
+    <row r="61" spans="2:4">
+      <c r="B61" s="12"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="12"/>
+    </row>
+    <row r="62" spans="2:4">
+      <c r="B62" s="12"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="2:4">
+      <c r="B63" s="12"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" spans="2:4">
+      <c r="B64" s="12"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="12"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="12"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="12"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="12"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="12"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="2:4">
+      <c r="B69" s="12"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="2:4">
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="2:4">
+      <c r="B71" s="12"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="2:4">
+      <c r="B72" s="12"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="12"/>
+    </row>
+    <row r="73" spans="2:4">
+      <c r="B73" s="12"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="2:4">
+      <c r="B74" s="12"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="12"/>
+    </row>
+    <row r="75" spans="2:4">
+      <c r="B75" s="12"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="12"/>
+    </row>
+    <row r="76" spans="2:4">
+      <c r="B76" s="12"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="12"/>
+    </row>
+    <row r="77" spans="2:4">
+      <c r="B77" s="12"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="12"/>
+    </row>
+    <row r="78" spans="2:4">
+      <c r="B78" s="12"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="12"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:B41"/>

</xml_diff>